<commit_message>
clase sobre pensamientos matamáticos lista.
</commit_message>
<xml_diff>
--- a/clases_2025_1/1_documentos_actas/parejas_practica_v.xlsx
+++ b/clases_2025_1/1_documentos_actas/parejas_practica_v.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\docencia\practica_v_dllo_pto_math_infancia\clases_2025_1\1_documentos_actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180B402A-12AF-49B4-A820-11BDC9C83E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2806DD-11E0-4BBC-8867-F0B74F9746E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>Grupo_1</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Primer  grado</t>
   </si>
   <si>
-    <t>grado primero</t>
-  </si>
-  <si>
     <t>Grado 1</t>
   </si>
   <si>
@@ -158,22 +155,35 @@
     <t>ItemGrupo</t>
   </si>
   <si>
-    <t>['Alvarez Perez Carlos Julio', '']</t>
-  </si>
-  <si>
     <t>Ítem</t>
+  </si>
+  <si>
+    <t>Nombres</t>
+  </si>
+  <si>
+    <t>['Alvarez Perez Carlos Julio', 'Sara Guerra']</t>
+  </si>
+  <si>
+    <t>["Yesika Martinez", "Xiomara López"]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -220,11 +230,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,17 +520,24 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="10.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
     <col min="3" max="3" width="36.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.33203125" customWidth="1"/>
     <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -532,9 +556,11 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" t="s">
+      <c r="B2" t="s">
         <v>5</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -550,7 +576,7 @@
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="C3" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
@@ -567,118 +593,122 @@
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" t="s">
-        <v>20</v>
-      </c>
       <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
         <v>30</v>
-      </c>
-      <c r="G7" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
         <v>21</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F9" t="s">
         <v>12</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
         <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
         <v>36</v>
       </c>
-      <c r="D12" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="F12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
         <v>1</v>
       </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
       <c r="E13" s="2"/>
+      <c r="F13" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
         <v>2</v>
       </c>
+      <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:7">
       <c r="A15">
         <v>3</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="4">
         <v>3</v>
       </c>
     </row>

</xml_diff>